<commit_message>
Hari Rabu, 15 Juli 2026, Melanjutkan progress untuk pembetulan periode dan semester
</commit_message>
<xml_diff>
--- a/siakad/public/document/template_import_biodata.xlsx
+++ b/siakad/public/document/template_import_biodata.xlsx
@@ -1,27 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Michael Setiawan\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC856715-2354-49DF-A26A-6B1472ECCE5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42022DCB-6F4D-4606-A3AA-6E2F67A88009}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Template Biodata" sheetId="1" r:id="rId1"/>
-    <sheet name="Panduan" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="108">
   <si>
     <t>nrp</t>
   </si>
@@ -221,94 +220,7 @@
     <t>nisn</t>
   </si>
   <si>
-    <t>Panduan Template Import Biodata</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>Isi data mulai baris 2 pada sheet Template Biodata.</t>
-  </si>
-  <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>Jangan ubah nama header, urutan kolom, atau menghapus kolom.</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>Format tanggal lahir dan last_update: YYYY-MM-DD.</t>
-  </si>
-  <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t>Kolom integer: tinggi, berat, anak_ke, jml_saudara, jml_saudara_tanggungan, kps.</t>
-  </si>
-  <si>
-    <t>5</t>
-  </si>
-  <si>
-    <t>Jenis kelamin hanya boleh: L atau P.</t>
-  </si>
-  <si>
-    <t>6</t>
-  </si>
-  <si>
-    <t>File import dapat berupa CSV, XLSX, atau XLS.</t>
-  </si>
-  <si>
-    <t>Kolom Kunci</t>
-  </si>
-  <si>
-    <t>Contoh</t>
-  </si>
-  <si>
-    <t>Keterangan</t>
-  </si>
-  <si>
-    <t>Wajib</t>
-  </si>
-  <si>
-    <t>31128888</t>
-  </si>
-  <si>
-    <t>Maksimal 8 karakter</t>
-  </si>
-  <si>
-    <t>Ya</t>
-  </si>
-  <si>
-    <t>2000-01-01</t>
-  </si>
-  <si>
-    <t>Format tanggal</t>
-  </si>
-  <si>
-    <t>Opsional</t>
-  </si>
-  <si>
-    <t>2026-06-30</t>
-  </si>
-  <si>
-    <t>nama@email.com</t>
-  </si>
-  <si>
-    <t>Format email valid</t>
-  </si>
-  <si>
     <t>L</t>
-  </si>
-  <si>
-    <t>L atau P</t>
-  </si>
-  <si>
-    <t>1234567890</t>
-  </si>
-  <si>
-    <t>Nomor NISN</t>
   </si>
   <si>
     <t>Ahmad Fauzi Pratama</t>
@@ -438,13 +350,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="2">
     <font>
-      <sz val="11"/>
-      <name val="Carlito"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <name val="Carlito"/>
     </font>
@@ -455,7 +362,7 @@
       <name val="Carlito"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -465,16 +372,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF1D4ED8"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF0F766E"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFDBEAFE"/>
       </patternFill>
     </fill>
   </fills>
@@ -490,23 +387,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -719,202 +606,202 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:66" ht="28.8" customHeight="1">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="2" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="2" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="2" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="2" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="2" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="2" t="s">
+      <c r="X1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="2" t="s">
+      <c r="Y1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="2" t="s">
+      <c r="Z1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="2" t="s">
+      <c r="AA1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" s="2" t="s">
+      <c r="AB1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="AC1" s="2" t="s">
+      <c r="AC1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="AD1" s="2" t="s">
+      <c r="AD1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="AE1" s="2" t="s">
+      <c r="AE1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="AF1" s="2" t="s">
+      <c r="AF1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="AG1" s="2" t="s">
+      <c r="AG1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="AH1" s="2" t="s">
+      <c r="AH1" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="AI1" s="2" t="s">
+      <c r="AI1" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="AJ1" s="2" t="s">
+      <c r="AJ1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="AK1" s="2" t="s">
+      <c r="AK1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="AL1" s="2" t="s">
+      <c r="AL1" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="AM1" s="2" t="s">
+      <c r="AM1" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="AN1" s="2" t="s">
+      <c r="AN1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="AO1" s="2" t="s">
+      <c r="AO1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="AP1" s="2" t="s">
+      <c r="AP1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="AQ1" s="2" t="s">
+      <c r="AQ1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="AR1" s="2" t="s">
+      <c r="AR1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="AS1" s="2" t="s">
+      <c r="AS1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="AT1" s="2" t="s">
+      <c r="AT1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="AU1" s="2" t="s">
+      <c r="AU1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="AV1" s="2" t="s">
+      <c r="AV1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="AW1" s="2" t="s">
+      <c r="AW1" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="AX1" s="2" t="s">
+      <c r="AX1" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="AY1" s="2" t="s">
+      <c r="AY1" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="AZ1" s="2" t="s">
+      <c r="AZ1" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="BA1" s="2" t="s">
+      <c r="BA1" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="BB1" s="2" t="s">
+      <c r="BB1" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="BC1" s="2" t="s">
+      <c r="BC1" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="BD1" s="2" t="s">
+      <c r="BD1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="BE1" s="2" t="s">
+      <c r="BE1" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="BF1" s="2" t="s">
+      <c r="BF1" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="BG1" s="2" t="s">
+      <c r="BG1" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="BH1" s="2" t="s">
+      <c r="BH1" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="BI1" s="2" t="s">
+      <c r="BI1" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="BJ1" s="2" t="s">
+      <c r="BJ1" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="BK1" s="2" t="s">
+      <c r="BK1" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="BL1" s="2" t="s">
+      <c r="BL1" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="BM1" s="2" t="s">
+      <c r="BM1" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="BN1" s="2" t="s">
+      <c r="BN1" s="1" t="s">
         <v>65</v>
       </c>
     </row>
@@ -923,15 +810,15 @@
         <v>31125555</v>
       </c>
       <c r="B2" t="s">
-        <v>96</v>
-      </c>
-      <c r="C2" s="5">
+        <v>67</v>
+      </c>
+      <c r="C2" s="2">
         <v>3578010000000000</v>
       </c>
       <c r="D2" t="s">
-        <v>97</v>
-      </c>
-      <c r="E2" s="6">
+        <v>68</v>
+      </c>
+      <c r="E2" s="3">
         <v>36713</v>
       </c>
       <c r="F2">
@@ -941,16 +828,16 @@
         <v>65</v>
       </c>
       <c r="H2" t="s">
-        <v>98</v>
+        <v>69</v>
       </c>
       <c r="I2" t="s">
-        <v>99</v>
+        <v>70</v>
       </c>
       <c r="J2" t="s">
-        <v>100</v>
+        <v>71</v>
       </c>
       <c r="K2" t="s">
-        <v>97</v>
+        <v>68</v>
       </c>
       <c r="L2">
         <v>60281</v>
@@ -962,19 +849,19 @@
         <v>81234567801</v>
       </c>
       <c r="O2" t="s">
-        <v>101</v>
+        <v>72</v>
       </c>
       <c r="P2" t="s">
-        <v>102</v>
+        <v>73</v>
       </c>
       <c r="Q2" t="s">
-        <v>103</v>
+        <v>74</v>
       </c>
       <c r="R2" t="s">
-        <v>104</v>
+        <v>75</v>
       </c>
       <c r="S2" t="s">
-        <v>105</v>
+        <v>76</v>
       </c>
       <c r="T2">
         <v>1</v>
@@ -986,31 +873,31 @@
         <v>1</v>
       </c>
       <c r="W2" t="s">
-        <v>106</v>
+        <v>77</v>
       </c>
       <c r="X2" t="s">
-        <v>107</v>
+        <v>78</v>
       </c>
       <c r="Y2" t="s">
-        <v>108</v>
+        <v>79</v>
       </c>
       <c r="Z2">
         <v>2018</v>
       </c>
       <c r="AA2" t="s">
-        <v>109</v>
+        <v>80</v>
       </c>
       <c r="AB2" t="s">
-        <v>110</v>
+        <v>81</v>
       </c>
       <c r="AC2" t="s">
-        <v>98</v>
+        <v>69</v>
       </c>
       <c r="AD2">
         <v>315678901</v>
       </c>
       <c r="AE2" t="s">
-        <v>97</v>
+        <v>68</v>
       </c>
       <c r="AF2">
         <v>60281</v>
@@ -1019,25 +906,25 @@
         <v>81234567802</v>
       </c>
       <c r="AH2" t="s">
-        <v>102</v>
+        <v>73</v>
       </c>
       <c r="AI2" t="s">
-        <v>111</v>
+        <v>82</v>
       </c>
       <c r="AJ2" t="s">
-        <v>112</v>
+        <v>83</v>
       </c>
       <c r="AK2" t="s">
-        <v>103</v>
+        <v>74</v>
       </c>
       <c r="AL2" t="s">
-        <v>113</v>
+        <v>84</v>
       </c>
       <c r="AM2" t="s">
-        <v>98</v>
+        <v>69</v>
       </c>
       <c r="AN2" t="s">
-        <v>97</v>
+        <v>68</v>
       </c>
       <c r="AO2">
         <v>60281</v>
@@ -1049,70 +936,70 @@
         <v>81234567803</v>
       </c>
       <c r="AR2" t="s">
-        <v>102</v>
+        <v>73</v>
       </c>
       <c r="AS2" t="s">
-        <v>114</v>
+        <v>85</v>
       </c>
       <c r="AT2" t="s">
-        <v>115</v>
+        <v>86</v>
       </c>
       <c r="AU2" t="s">
-        <v>103</v>
+        <v>74</v>
       </c>
       <c r="AV2" t="s">
-        <v>116</v>
+        <v>87</v>
       </c>
       <c r="AW2" t="s">
-        <v>116</v>
+        <v>87</v>
       </c>
       <c r="AX2" t="s">
-        <v>116</v>
+        <v>87</v>
       </c>
       <c r="AY2" t="s">
-        <v>116</v>
+        <v>87</v>
       </c>
       <c r="AZ2" t="s">
-        <v>116</v>
+        <v>87</v>
       </c>
       <c r="BA2" t="s">
-        <v>116</v>
+        <v>87</v>
       </c>
       <c r="BB2" t="s">
-        <v>116</v>
+        <v>87</v>
       </c>
       <c r="BC2" t="s">
-        <v>116</v>
+        <v>87</v>
       </c>
       <c r="BD2" t="s">
-        <v>116</v>
+        <v>87</v>
       </c>
       <c r="BE2" t="s">
-        <v>116</v>
+        <v>87</v>
       </c>
       <c r="BF2" t="s">
-        <v>117</v>
+        <v>88</v>
       </c>
       <c r="BG2">
         <v>0</v>
       </c>
       <c r="BH2" t="s">
-        <v>118</v>
+        <v>89</v>
       </c>
       <c r="BI2" t="s">
-        <v>117</v>
+        <v>88</v>
       </c>
       <c r="BJ2" t="s">
-        <v>117</v>
-      </c>
-      <c r="BK2" s="6">
+        <v>88</v>
+      </c>
+      <c r="BK2" s="3">
         <v>46174</v>
       </c>
       <c r="BL2" t="s">
-        <v>119</v>
+        <v>90</v>
       </c>
       <c r="BM2" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="BN2">
         <v>12345678</v>
@@ -1123,15 +1010,15 @@
         <v>31126666</v>
       </c>
       <c r="B3" t="s">
-        <v>120</v>
-      </c>
-      <c r="C3" s="5">
+        <v>91</v>
+      </c>
+      <c r="C3" s="2">
         <v>3578030000000000</v>
       </c>
       <c r="D3" t="s">
-        <v>121</v>
-      </c>
-      <c r="E3" s="6">
+        <v>92</v>
+      </c>
+      <c r="E3" s="3">
         <v>36714</v>
       </c>
       <c r="F3">
@@ -1141,16 +1028,16 @@
         <v>50</v>
       </c>
       <c r="H3" t="s">
-        <v>122</v>
+        <v>93</v>
       </c>
       <c r="I3" t="s">
-        <v>123</v>
+        <v>94</v>
       </c>
       <c r="J3" t="s">
-        <v>124</v>
+        <v>95</v>
       </c>
       <c r="K3" t="s">
-        <v>121</v>
+        <v>92</v>
       </c>
       <c r="L3">
         <v>65141</v>
@@ -1162,19 +1049,19 @@
         <v>81234567804</v>
       </c>
       <c r="O3" t="s">
-        <v>125</v>
+        <v>96</v>
       </c>
       <c r="P3" t="s">
-        <v>126</v>
+        <v>97</v>
       </c>
       <c r="Q3" t="s">
-        <v>103</v>
+        <v>74</v>
       </c>
       <c r="R3" t="s">
-        <v>104</v>
+        <v>75</v>
       </c>
       <c r="S3" t="s">
-        <v>127</v>
+        <v>98</v>
       </c>
       <c r="T3">
         <v>2</v>
@@ -1186,31 +1073,31 @@
         <v>1</v>
       </c>
       <c r="W3" t="s">
-        <v>128</v>
+        <v>99</v>
       </c>
       <c r="X3" t="s">
-        <v>107</v>
+        <v>78</v>
       </c>
       <c r="Y3" t="s">
-        <v>129</v>
+        <v>100</v>
       </c>
       <c r="Z3">
         <v>2018</v>
       </c>
       <c r="AA3" t="s">
-        <v>130</v>
+        <v>101</v>
       </c>
       <c r="AB3" t="s">
-        <v>131</v>
+        <v>102</v>
       </c>
       <c r="AC3" t="s">
-        <v>122</v>
+        <v>93</v>
       </c>
       <c r="AD3">
         <v>341234567</v>
       </c>
       <c r="AE3" t="s">
-        <v>121</v>
+        <v>92</v>
       </c>
       <c r="AF3">
         <v>65141</v>
@@ -1219,25 +1106,25 @@
         <v>81234567805</v>
       </c>
       <c r="AH3" t="s">
-        <v>126</v>
+        <v>97</v>
       </c>
       <c r="AI3" t="s">
-        <v>132</v>
+        <v>103</v>
       </c>
       <c r="AJ3" t="s">
-        <v>112</v>
+        <v>83</v>
       </c>
       <c r="AK3" t="s">
-        <v>103</v>
+        <v>74</v>
       </c>
       <c r="AL3" t="s">
-        <v>133</v>
+        <v>104</v>
       </c>
       <c r="AM3" t="s">
-        <v>122</v>
+        <v>93</v>
       </c>
       <c r="AN3" t="s">
-        <v>121</v>
+        <v>92</v>
       </c>
       <c r="AO3">
         <v>65141</v>
@@ -1249,70 +1136,70 @@
         <v>81234567806</v>
       </c>
       <c r="AR3" t="s">
-        <v>126</v>
+        <v>97</v>
       </c>
       <c r="AS3" t="s">
-        <v>134</v>
+        <v>105</v>
       </c>
       <c r="AT3" t="s">
-        <v>112</v>
+        <v>83</v>
       </c>
       <c r="AU3" t="s">
-        <v>103</v>
+        <v>74</v>
       </c>
       <c r="AV3" t="s">
-        <v>116</v>
+        <v>87</v>
       </c>
       <c r="AW3" t="s">
-        <v>116</v>
+        <v>87</v>
       </c>
       <c r="AX3" t="s">
-        <v>116</v>
+        <v>87</v>
       </c>
       <c r="AY3" t="s">
-        <v>116</v>
+        <v>87</v>
       </c>
       <c r="AZ3" t="s">
-        <v>116</v>
+        <v>87</v>
       </c>
       <c r="BA3" t="s">
-        <v>116</v>
+        <v>87</v>
       </c>
       <c r="BB3" t="s">
-        <v>116</v>
+        <v>87</v>
       </c>
       <c r="BC3" t="s">
-        <v>116</v>
+        <v>87</v>
       </c>
       <c r="BD3" t="s">
-        <v>116</v>
+        <v>87</v>
       </c>
       <c r="BE3" t="s">
-        <v>116</v>
+        <v>87</v>
       </c>
       <c r="BF3" t="s">
-        <v>117</v>
+        <v>88</v>
       </c>
       <c r="BG3">
         <v>1</v>
       </c>
       <c r="BH3" t="s">
-        <v>118</v>
+        <v>89</v>
       </c>
       <c r="BI3" t="s">
-        <v>117</v>
+        <v>88</v>
       </c>
       <c r="BJ3" t="s">
-        <v>117</v>
-      </c>
-      <c r="BK3" s="6">
+        <v>88</v>
+      </c>
+      <c r="BK3" s="3">
         <v>46175</v>
       </c>
       <c r="BL3" t="s">
-        <v>135</v>
+        <v>106</v>
       </c>
       <c r="BM3" t="s">
-        <v>136</v>
+        <v>107</v>
       </c>
       <c r="BN3">
         <v>12345679</v>
@@ -1321,189 +1208,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:D16"/>
-  <sheetFormatPr defaultRowHeight="13.8"/>
-  <cols>
-    <col min="1" max="1" width="16" customWidth="1"/>
-    <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="3" max="3" width="30" customWidth="1"/>
-    <col min="4" max="4" width="10" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" ht="22.35" customHeight="1">
-      <c r="A1" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-    </row>
-    <row r="3" spans="1:4" ht="41.4">
-      <c r="A3" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
-    </row>
-    <row r="4" spans="1:4" ht="55.2">
-      <c r="A4" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-    </row>
-    <row r="5" spans="1:4" ht="41.4">
-      <c r="A5" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-    </row>
-    <row r="6" spans="1:4" ht="69">
-      <c r="A6" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
-    </row>
-    <row r="7" spans="1:4" ht="27.6">
-      <c r="A7" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-    </row>
-    <row r="8" spans="1:4" ht="41.4">
-      <c r="A8" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
-    </row>
-    <row r="10" spans="1:4">
-      <c r="A10" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4">
-      <c r="A11" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4">
-      <c r="A12" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4">
-      <c r="A13" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4">
-      <c r="A14" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="D14" s="3" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4">
-      <c r="A15" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="D15" s="3" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4">
-      <c r="A16" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="D16" s="3" t="s">
-        <v>85</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>